<commit_message>
Coffee Cart (EN): arreglos de la revisión en los 5 entregables (B1 comparativa cart/trailer/truck en el Word, M1-M7, m1-m15, m21-m24); G1-G9 verdes, regresión 39/39
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/coffee-cart-business-plan/coffee-cart-financial-projections.xlsx
+++ b/astro-site/public/dl/coffee-cart-business-plan/coffee-cart-financial-projections.xlsx
@@ -814,8 +814,8 @@
         <v>13.608</v>
       </c>
       <c r="C9" t="str">
-        <f>IFERROR("Price per guest excl. sales tax plus the weighted sales tax of your sales lines ("&amp;TEXT(SUMPRODUCT('3-Year P&amp;L'!$E$10:$E$11,'3-Year P&amp;L'!$G$10:$G$11)*100,"0")&amp;"%), rounded. In the US the quote adds sales tax on top, and many states tax the whole catering invoice (coffee service, baristas, add-ons and travel); in the UK, VAT is included in the price.","")</f>
-        <v>Price per guest excl. sales tax plus the weighted sales tax of your sales lines (8%), rounded. In the US the quote adds sales tax on top, and many states tax the whole catering invoice (coffee service, baristas, add-ons and travel); in the UK, VAT is included in the price.</v>
+        <f>IFERROR("Price per guest excl. sales tax plus the weighted sales tax of your sales lines ("&amp;TEXT(SUMPRODUCT('3-Year P&amp;L'!$E$10:$E$11,'3-Year P&amp;L'!$G$10:$G$11)*100,"0")&amp;"%), rounded. In the US the quote adds sales tax on top, and many states tax the whole catering invoice (coffee service, baristas and add-ons; in some states, travel too); in the UK, VAT is included in the price.","")</f>
+        <v>Price per guest excl. sales tax plus the weighted sales tax of your sales lines (8%), rounded. In the US the quote adds sales tax on top, and many states tax the whole catering invoice (coffee service, baristas and add-ons; in some states, travel too); in the UK, VAT is included in the price.</v>
       </c>
     </row>
     <row r="10">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Example: 21% federal rate for a C corporation plus state tax, rounded to 25%. If you operate as a sole proprietorship, LLC taxed as a pass-through or S corporation, the business itself pays 0% here and you pay tax on the profit personally: set this to 0 and budget for your personal tax separately. The model applies this rate to the first two years with positive taxable income</t>
+          <t>Example: 21% federal rate for a C corporation plus state tax, rounded to 25%. If you operate as a sole proprietorship, LLC taxed as a pass-through or S corporation, the business itself pays 0% here and you pay tax on the profit personally: set this to 0 and budget for your personal tax separately, or keep it as a reserve for your personal tax, as the Word plan does. The model applies this rate to the first two years with positive taxable income</t>
         </is>
       </c>
     </row>
@@ -1225,14 +1225,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Example rate: state + local sales tax combined, applied to the whole invoice (coffee service, baristas, add-ons and travel). Hosted events are usually taxed as catering; at festivals and markets you collect it drink by drink and may need a permit where you sell. Rates and rules vary widely by state and city: look up yours. UK: 20% VAT applies to catering for events and functions (VAT Notice 709/1).</t>
+          <t>Example rate: state + local sales tax combined, applied to the whole invoice (coffee service, baristas and add-ons, and in some states the travel fee). Hosted events are usually taxed as catering; at festivals and markets you collect it drink by drink and may need a permit where you sell. Rates and rules vary widely by state and city: look up yours. UK: 20% VAT applies to catering for events and functions (VAT Notice 709/1).</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Sales tax rate on alcohol sold (licensed only)</t>
+          <t>Sales tax rate on alcohol (not used: no alcohol in this plan)</t>
         </is>
       </c>
       <c r="B40" s="63" t="n">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Same example rate as above. Some states add separate liquor taxes: include them here if they apply to you. Alcohol served on site has its own rate in the sales tax breakdown block, further down. Utilities, equipment and services are handled in the cell below</t>
+          <t>Not used: this plan sells no alcohol (row 62 is 0%). If you ever sell alcohol under a license, enter its rate here and add any state liquor taxes.</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Average days between the event and the money in your bank. Hosts usually pay a retainer of 30-50% when they book the date (grindkit.app) and the balance 14 days before the event, while companies often pay at 15-30 days, so the example sits in between. Raise it if your clients pay later. The workbook does not model deposits: they improve your real cash flow.</t>
+          <t>Average days between the event and the money in your bank. Hosts usually pay a retainer of 30-50% when they book the date (grindkit.app) and the balance 14 days before the event, while companies often pay at 15-30 days, so the example sits in between. Raise it if your clients pay later. The workbook does not model retainers: they improve your real cash flow.</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6295,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="74.75" customHeight="1">
+    <row r="45" ht="89.75" customHeight="1">
       <c r="A45" s="58" t="inlineStr">
         <is>
           <t>Income tax</t>
@@ -6313,7 +6313,7 @@
       </c>
       <c r="D45" s="17" t="inlineStr">
         <is>
-          <t>A loss in one year reduces taxable profit in later years. The model offsets losses fully as a simplification (federal rules cap the offset at 80% of taxable income). If you operate as a pass-through (sole proprietorship or LLC), set the rate to 0 and budget your personal tax separately.</t>
+          <t>A loss in one year reduces taxable profit in later years. The model offsets losses fully as a simplification (federal rules cap the offset at 80% of taxable income). If you operate as a pass-through (sole proprietorship or LLC), set the rate to 0 and budget your personal tax separately, or keep it as a reserve for that tax, as the Word plan does.</t>
         </is>
       </c>
     </row>
@@ -6610,7 +6610,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="45" customHeight="1">
+    <row r="61" ht="59.75" customHeight="1">
       <c r="A61" t="inlineStr">
         <is>
           <t>Startup cost of a coffee cart</t>
@@ -6618,17 +6618,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>$5,000-25,000 for a cart; a 2-group machine about $8,500</t>
+          <t>$4,000-25,000 for the cart; $16,600-49,000 all in ($24,000 typical); a 2-group machine about $8,500</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>cart-king.com; Kit estimate</t>
+          <t>cart-king.com; Kit estimate (machine)</t>
         </is>
       </c>
       <c r="D61" s="17" t="inlineStr">
         <is>
-          <t>Cart-king.com lists a typical cart at $24,000 and a premium one at $49,000. The $5,000-25,000 range and the machine price (store price) are Kit estimates.</t>
+          <t>Cart-king.com puts the cart itself at $4,000-25,000 (basic new to custom premium) and a complete single-cart setup at about $16,600-49,000, with $24,000 typical. The machine price is a store price (Kit estimate).</t>
         </is>
       </c>
     </row>
@@ -6742,7 +6742,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="59.75" customHeight="1">
+    <row r="67" ht="74.75" customHeight="1">
       <c r="A67" t="inlineStr">
         <is>
           <t>Insurance</t>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="D67" s="17" t="inlineStr">
         <is>
-          <t>Insureon averages for businesses under 5 employees: general liability, BOP, workers' comp and commercial auto. Your quotes will differ. Venues usually ask for unlimited additional insureds, and your commercial auto must cover the trailer.</t>
+          <t>Insureon averages for businesses under 5 employees: general liability, BOP, workers' comp and commercial auto. Your quotes will differ, and the kit's example is a lean budget: get quotes. Venues usually ask for unlimited additional insureds, and your commercial auto must cover the trailer.</t>
         </is>
       </c>
     </row>
@@ -7656,7 +7656,7 @@
       </c>
       <c r="O16" s="28" t="inlineStr">
         <is>
-          <t>Each sales line at ITS OWN rate, read from the sales tax column of the P&amp;L (alcohol to go has its own rate cell in the Assumptions tab)</t>
+          <t>Each sales line at ITS OWN rate, read from the sales tax column of the P&amp;L</t>
         </is>
       </c>
     </row>

</xml_diff>